<commit_message>
Working Full Thermal Distribtion solve - scaling issues still present
</commit_message>
<xml_diff>
--- a/data_structure.xlsx
+++ b/data_structure.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="54" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="53" uniqueCount="32">
   <si>
     <t>n_element</t>
   </si>
@@ -7441,7 +7441,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="0">
         <v>7</v>
@@ -7449,10 +7449,12 @@
       <c r="C10" s="0">
         <v>8</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="0"/>
+      <c r="D10" s="0">
+        <v>22</v>
+      </c>
+      <c r="E10" s="0">
+        <v>20</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">

</xml_diff>